<commit_message>
Introduce segmented SQLite workflow state and wire policy tooling to database-backed tasks
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$36</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="798" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="113">
   <si>
     <t>candidate_id</t>
   </si>
@@ -329,6 +329,33 @@
   </si>
   <si>
     <t>35359</t>
+  </si>
+  <si>
+    <t>2026-02-18T21:30:05Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-sqlite-state-tooling</t>
+  </si>
+  <si>
+    <t>2026-02-18T21:29:28.639788139Z</t>
+  </si>
+  <si>
+    <t>Promote the SQLite-backed workflow state model introduced in `afp-converter` into `pz-boilerplate-intelliJ` so project-management automation defaults to database-backed tooling instead of ad-hoc scripts.</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>860</t>
+  </si>
+  <si>
+    <t>444</t>
+  </si>
+  <si>
+    <t>575</t>
+  </si>
+  <si>
+    <t>829</t>
   </si>
 </sst>
 </file>
@@ -373,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -461,7 +488,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3">
@@ -505,7 +532,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +576,7 @@
         <v>24</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5">
@@ -593,15 +620,15 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>100</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>16</v>
@@ -610,45 +637,89 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>107</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="N6" t="s" s="0">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E7" t="s" s="0">
         <v>34</v>
       </c>
-      <c r="F6" t="s" s="0">
+      <c r="F7" t="s" s="0">
         <v>35</v>
       </c>
-      <c r="G6" t="s" s="0">
+      <c r="G7" t="s" s="0">
         <v>36</v>
       </c>
-      <c r="H6" t="s" s="0">
+      <c r="H7" t="s" s="0">
         <v>21</v>
       </c>
-      <c r="I6" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="J6" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="K6" t="s" s="0">
-        <v>22</v>
-      </c>
-      <c r="L6" t="s" s="0">
+      <c r="I7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L7" t="s" s="0">
         <v>98</v>
       </c>
-      <c r="M6" t="s" s="0">
+      <c r="M7" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="N6" t="s" s="0">
-        <v>100</v>
+      <c r="N7" t="s" s="0">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N6"/>
+  <autoFilter ref="A1:N7"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -950,46 +1021,46 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B28" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>59</v>
+        <v>109</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B29" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>60</v>
+        <v>110</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B30" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>61</v>
+        <v>111</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B31" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>46</v>
+        <v>112</v>
       </c>
     </row>
     <row r="32">
@@ -997,14 +1068,58 @@
         <v>32</v>
       </c>
       <c r="B32" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C33" t="s" s="0">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C34" t="s" s="0">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C35" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B36" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="C32" t="s" s="0">
+      <c r="C36" t="s" s="0">
         <v>63</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C32"/>
+  <autoFilter ref="A1:C36"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Enforce product-management boundary gate and expand governance/state auditing workflow
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$52</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="140">
   <si>
     <t>candidate_id</t>
   </si>
@@ -356,6 +356,87 @@
   </si>
   <si>
     <t>829</t>
+  </si>
+  <si>
+    <t>2026-02-18T21:49:44Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-governance-events-workbook</t>
+  </si>
+  <si>
+    <t>2026-02-18T21:49:35.000160283Z</t>
+  </si>
+  <si>
+    <t>Add explicit policy-governance event tracking (CSV + generated XLSX + build task) to the boilerplate framework so future agents must leave an auditable governance trail.</t>
+  </si>
+  <si>
+    <t>454</t>
+  </si>
+  <si>
+    <t>116</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>893</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:02:21Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-governance-alerts-trust-sot</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:02:11.800080022Z</t>
+  </si>
+  <si>
+    <t>Promote constitutional governance-breach visibility and trust-grant logging into boilerplate workflow, backed by SQLite state as single source of truth.</t>
+  </si>
+  <si>
+    <t>443</t>
+  </si>
+  <si>
+    <t>828</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:10:17Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-vcs-file-discipline-ledger</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:10:08.096095749Z</t>
+  </si>
+  <si>
+    <t>Add mirrored version-control/file-discipline ledgering to the SQLite project state workflow.</t>
+  </si>
+  <si>
+    <t>411</t>
+  </si>
+  <si>
+    <t>797</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:16:18Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-product-management-boundary-gate</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:16:07.03604653Z</t>
+  </si>
+  <si>
+    <t>Add a hard verification gate to prevent product modules from referencing project-management tooling/state.</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>296</t>
+  </si>
+  <si>
+    <t>617</t>
   </si>
 </sst>
 </file>
@@ -400,7 +481,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -488,7 +569,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3">
@@ -532,15 +613,15 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>15</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>16</v>
@@ -549,16 +630,16 @@
         <v>17</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>18</v>
+        <v>123</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>19</v>
+        <v>124</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>21</v>
+        <v>108</v>
       </c>
       <c r="I4" t="s" s="0">
         <v>22</v>
@@ -570,21 +651,21 @@
         <v>22</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="M4" t="s" s="0">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>16</v>
@@ -593,16 +674,16 @@
         <v>17</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>28</v>
+        <v>115</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>29</v>
+        <v>116</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>21</v>
+        <v>108</v>
       </c>
       <c r="I5" t="s" s="0">
         <v>22</v>
@@ -614,21 +695,21 @@
         <v>22</v>
       </c>
       <c r="L5" t="s" s="0">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="M5" t="s" s="0">
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>105</v>
+        <v>134</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>105</v>
+        <v>134</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>16</v>
@@ -637,10 +718,10 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>106</v>
+        <v>135</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>107</v>
+        <v>136</v>
       </c>
       <c r="G6" t="s" s="0">
         <v>22</v>
@@ -661,18 +742,18 @@
         <v>23</v>
       </c>
       <c r="M6" t="s" s="0">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>16</v>
@@ -681,13 +762,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="H7" t="s" s="0">
         <v>21</v>
@@ -708,18 +789,194 @@
         <v>24</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>104</v>
+        <v>133</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L8" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="M8" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="N8" t="s" s="0">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>106</v>
+      </c>
+      <c r="F9" t="s" s="0">
+        <v>107</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J9" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K9" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L9" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M9" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="N9" t="s" s="0">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="F10" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K10" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L10" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M10" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="N10" t="s" s="0">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="G11" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="H11" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L11" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="M11" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="N11" t="s" s="0">
+        <v>133</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N7"/>
+  <autoFilter ref="A1:N11"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C52"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -889,237 +1146,413 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="B16" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>40</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="B17" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>42</v>
+        <v>118</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>44</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>14</v>
+        <v>122</v>
       </c>
       <c r="B19" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>46</v>
+        <v>126</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>14</v>
+        <v>114</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>48</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>49</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>50</v>
+        <v>119</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>26</v>
+        <v>114</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>51</v>
+        <v>120</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>52</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>54</v>
+        <v>118</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>56</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>58</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B28" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>109</v>
+        <v>40</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B29" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>110</v>
+        <v>42</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B30" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>111</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>112</v>
+        <v>46</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>59</v>
+        <v>48</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>60</v>
+        <v>49</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>61</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>46</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C36" t="s" s="0">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="C37" t="s" s="0">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C38" t="s" s="0">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="C39" t="s" s="0">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C40" t="s" s="0">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C41" t="s" s="0">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C42" t="s" s="0">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C43" t="s" s="0">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C44" t="s" s="0">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C45" t="s" s="0">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C46" t="s" s="0">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C47" t="s" s="0">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="B36" t="s" s="0">
+      <c r="B48" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C48" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C49" t="s" s="0">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C50" t="s" s="0">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C51" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B52" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="C36" t="s" s="0">
+      <c r="C52" t="s" s="0">
         <v>63</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C36"/>
+  <autoFilter ref="A1:C52"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: normalize PM realm workflow and add boilerplate roll-up package
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$52</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$65</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2088" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3930" uniqueCount="174">
   <si>
     <t>candidate_id</t>
   </si>
@@ -437,6 +437,108 @@
   </si>
   <si>
     <t>617</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:27:36Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-unified-framework-rollup</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:26:51.532573445Z</t>
+  </si>
+  <si>
+    <t>Single consolidated transfer package for `pz-boilerplate-intelliJ` that supersedes all current review-state packages from this cycle.</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>446</t>
+  </si>
+  <si>
+    <t>390</t>
+  </si>
+  <si>
+    <t>1430</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:38:34Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-managed-tooling-registration-gate</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:38:24.013588086Z</t>
+  </si>
+  <si>
+    <t>Add constitutional managed-tooling discipline and build enforcement so untracked project-management tooling cannot bypass workflow controls.</t>
+  </si>
+  <si>
+    <t>342</t>
+  </si>
+  <si>
+    <t>606</t>
+  </si>
+  <si>
+    <t>2026-02-18T22:43:20Z</t>
+  </si>
+  <si>
+    <t>1573</t>
+  </si>
+  <si>
+    <t>2026-02-18T23:37:27Z</t>
+  </si>
+  <si>
+    <t>2026-02-18-pm-realm-console-sql-rules-rollup</t>
+  </si>
+  <si>
+    <t>2026-02-18T23:36:34.923252375Z</t>
+  </si>
+  <si>
+    <t>Single roll-up transfer package for `pz-boilerplate-intelliJ` that consolidates the latest project-management framework changes:</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>785</t>
+  </si>
+  <si>
+    <t>863</t>
+  </si>
+  <si>
+    <t>436</t>
+  </si>
+  <si>
+    <t>1368</t>
+  </si>
+  <si>
+    <t>patches/0001-pm-realm-console-sql-rules-rollup.patch</t>
+  </si>
+  <si>
+    <t>152465</t>
+  </si>
+  <si>
+    <t>2026-02-18T23:53:29Z</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>978</t>
+  </si>
+  <si>
+    <t>992</t>
+  </si>
+  <si>
+    <t>566</t>
+  </si>
+  <si>
+    <t>1622</t>
+  </si>
+  <si>
+    <t>159406</t>
   </si>
 </sst>
 </file>
@@ -481,7 +583,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -569,7 +671,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3">
@@ -607,13 +709,13 @@
         <v>22</v>
       </c>
       <c r="L3" t="s" s="0">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="M3" t="s" s="0">
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="4">
@@ -651,13 +753,13 @@
         <v>22</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="M4" t="s" s="0">
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5">
@@ -695,21 +797,21 @@
         <v>22</v>
       </c>
       <c r="L5" t="s" s="0">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="M5" t="s" s="0">
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="C6" t="s" s="0">
         <v>16</v>
@@ -718,10 +820,10 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="G6" t="s" s="0">
         <v>22</v>
@@ -739,21 +841,21 @@
         <v>22</v>
       </c>
       <c r="L6" t="s" s="0">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="M6" t="s" s="0">
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>15</v>
+        <v>157</v>
       </c>
       <c r="C7" t="s" s="0">
         <v>16</v>
@@ -762,13 +864,13 @@
         <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>18</v>
+        <v>158</v>
       </c>
       <c r="F7" t="s" s="0">
-        <v>19</v>
+        <v>159</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H7" t="s" s="0">
         <v>21</v>
@@ -783,21 +885,21 @@
         <v>22</v>
       </c>
       <c r="L7" t="s" s="0">
-        <v>98</v>
+        <v>23</v>
       </c>
       <c r="M7" t="s" s="0">
-        <v>24</v>
+        <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>27</v>
+        <v>134</v>
       </c>
       <c r="C8" t="s" s="0">
         <v>16</v>
@@ -806,16 +908,16 @@
         <v>17</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>28</v>
+        <v>135</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>29</v>
+        <v>136</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>21</v>
+        <v>108</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>22</v>
@@ -830,18 +932,18 @@
         <v>98</v>
       </c>
       <c r="M8" t="s" s="0">
-        <v>31</v>
+        <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>105</v>
+        <v>15</v>
       </c>
       <c r="C9" t="s" s="0">
         <v>16</v>
@@ -850,16 +952,16 @@
         <v>17</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>106</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>107</v>
+        <v>19</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="I9" t="s" s="0">
         <v>22</v>
@@ -871,21 +973,21 @@
         <v>22</v>
       </c>
       <c r="L9" t="s" s="0">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="M9" t="s" s="0">
-        <v>89</v>
+        <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>128</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s" s="0">
         <v>16</v>
@@ -894,16 +996,16 @@
         <v>17</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>129</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>130</v>
+        <v>29</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>108</v>
+        <v>21</v>
       </c>
       <c r="I10" t="s" s="0">
         <v>22</v>
@@ -915,21 +1017,21 @@
         <v>22</v>
       </c>
       <c r="L10" t="s" s="0">
-        <v>23</v>
+        <v>98</v>
       </c>
       <c r="M10" t="s" s="0">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>133</v>
+        <v>167</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>33</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s" s="0">
         <v>16</v>
@@ -938,16 +1040,16 @@
         <v>17</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>34</v>
+        <v>106</v>
       </c>
       <c r="F11" t="s" s="0">
-        <v>35</v>
+        <v>107</v>
       </c>
       <c r="G11" t="s" s="0">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="H11" t="s" s="0">
-        <v>21</v>
+        <v>108</v>
       </c>
       <c r="I11" t="s" s="0">
         <v>22</v>
@@ -962,21 +1064,153 @@
         <v>98</v>
       </c>
       <c r="M11" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="N11" t="s" s="0">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>142</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>143</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H12" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K12" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L12" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="M12" t="s" s="0">
+        <v>144</v>
+      </c>
+      <c r="N12" t="s" s="0">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>129</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>130</v>
+      </c>
+      <c r="G13" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H13" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I13" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J13" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K13" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L13" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="M13" t="s" s="0">
+        <v>89</v>
+      </c>
+      <c r="N13" t="s" s="0">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="G14" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="H14" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="I14" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J14" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K14" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L14" t="s" s="0">
+        <v>98</v>
+      </c>
+      <c r="M14" t="s" s="0">
         <v>24</v>
       </c>
-      <c r="N11" t="s" s="0">
-        <v>133</v>
+      <c r="N14" t="s" s="0">
+        <v>167</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N11"/>
+  <autoFilter ref="A1:N14"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C52"/>
+  <dimension ref="A1:C65"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1234,18 +1468,18 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="B24" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>138</v>
+        <v>152</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="B25" t="s" s="0">
         <v>41</v>
@@ -1256,7 +1490,7 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="B26" t="s" s="0">
         <v>43</v>
@@ -1267,292 +1501,435 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>134</v>
+        <v>149</v>
       </c>
       <c r="B27" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>139</v>
+        <v>153</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="B28" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>40</v>
+        <v>169</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="B29" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>42</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="B30" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>44</v>
+        <v>171</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="B31" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>46</v>
+        <v>172</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>14</v>
+        <v>157</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>47</v>
+        <v>165</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>48</v>
+        <v>173</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B33" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>49</v>
+        <v>138</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B34" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>50</v>
+        <v>118</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B35" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>51</v>
+        <v>119</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>26</v>
+        <v>134</v>
       </c>
       <c r="B36" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>52</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>54</v>
+        <v>40</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>58</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>109</v>
+        <v>46</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>105</v>
+        <v>14</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s" s="0">
-        <v>110</v>
+        <v>48</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C42" t="s" s="0">
-        <v>111</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>105</v>
+        <v>26</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C43" t="s" s="0">
-        <v>112</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>131</v>
+        <v>51</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>118</v>
+        <v>52</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>119</v>
+        <v>54</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>128</v>
+        <v>26</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>132</v>
+        <v>56</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>39</v>
+        <v>57</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>60</v>
+        <v>109</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>61</v>
+        <v>110</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>32</v>
+        <v>105</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>46</v>
+        <v>111</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
+        <v>105</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C52" t="s" s="0">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C53" t="s" s="0">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C54" t="s" s="0">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C55" t="s" s="0">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s" s="0">
+        <v>141</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C56" t="s" s="0">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C57" t="s" s="0">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C58" t="s" s="0">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C59" t="s" s="0">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s" s="0">
+        <v>128</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C60" t="s" s="0">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s" s="0">
         <v>32</v>
       </c>
-      <c r="B52" t="s" s="0">
+      <c r="B61" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C61" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C62" t="s" s="0">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C63" t="s" s="0">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C64" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B65" t="s" s="0">
         <v>62</v>
       </c>
-      <c r="C52" t="s" s="0">
+      <c r="C65" t="s" s="0">
         <v>63</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C52"/>
+  <autoFilter ref="A1:C65"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: move boilerplate packages to third realm and add convergence handoff
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$70</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3930" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4350" uniqueCount="207">
   <si>
     <t>candidate_id</t>
   </si>
@@ -539,6 +539,105 @@
   </si>
   <si>
     <t>159406</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.460249676Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:11:32Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.418877023Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.433450584Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.428495648Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.463930826Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.454837241Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.441698882Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.445724823Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.424861664Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.409969312Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.450678009Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.413832629Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.437973523Z</t>
+  </si>
+  <si>
+    <t>2026-02-19-fresh-instance-convergence-eval</t>
+  </si>
+  <si>
+    <t>2026-02-19T00:09:06.470757755Z</t>
+  </si>
+  <si>
+    <t>Provide a deterministic handoff pack for a fresh AI instance to:</t>
+  </si>
+  <si>
+    <t>348</t>
+  </si>
+  <si>
+    <t>2665</t>
+  </si>
+  <si>
+    <t>551</t>
+  </si>
+  <si>
+    <t>1265</t>
+  </si>
+  <si>
+    <t>505</t>
+  </si>
+  <si>
+    <t>999</t>
+  </si>
+  <si>
+    <t>573</t>
+  </si>
+  <si>
+    <t>642</t>
+  </si>
+  <si>
+    <t>515</t>
+  </si>
+  <si>
+    <t>423</t>
+  </si>
+  <si>
+    <t>667</t>
+  </si>
+  <si>
+    <t>781</t>
+  </si>
+  <si>
+    <t>comparison-checklist.md</t>
+  </si>
+  <si>
+    <t>1345</t>
+  </si>
+  <si>
+    <t>810</t>
+  </si>
+  <si>
+    <t>1680</t>
   </si>
 </sst>
 </file>
@@ -583,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N14"/>
+  <dimension ref="A1:N15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -644,7 +743,7 @@
         <v>17</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>66</v>
+        <v>174</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>67</v>
@@ -671,7 +770,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="3">
@@ -688,7 +787,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>86</v>
+        <v>176</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>87</v>
@@ -715,7 +814,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4">
@@ -732,7 +831,7 @@
         <v>17</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>123</v>
+        <v>177</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>124</v>
@@ -759,7 +858,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5">
@@ -776,7 +875,7 @@
         <v>17</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>115</v>
+        <v>178</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>116</v>
@@ -803,7 +902,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6">
@@ -820,7 +919,7 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>150</v>
+        <v>179</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>151</v>
@@ -847,7 +946,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7">
@@ -864,7 +963,7 @@
         <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>158</v>
+        <v>180</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>159</v>
@@ -891,7 +990,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8">
@@ -908,7 +1007,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>135</v>
+        <v>181</v>
       </c>
       <c r="F8" t="s" s="0">
         <v>136</v>
@@ -935,7 +1034,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9">
@@ -952,7 +1051,7 @@
         <v>17</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>18</v>
+        <v>182</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>19</v>
@@ -979,7 +1078,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="10">
@@ -996,7 +1095,7 @@
         <v>17</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>28</v>
+        <v>183</v>
       </c>
       <c r="F10" t="s" s="0">
         <v>29</v>
@@ -1023,7 +1122,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11">
@@ -1040,7 +1139,7 @@
         <v>17</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>106</v>
+        <v>184</v>
       </c>
       <c r="F11" t="s" s="0">
         <v>107</v>
@@ -1067,7 +1166,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="12">
@@ -1084,7 +1183,7 @@
         <v>17</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>142</v>
+        <v>185</v>
       </c>
       <c r="F12" t="s" s="0">
         <v>143</v>
@@ -1111,7 +1210,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="13">
@@ -1128,7 +1227,7 @@
         <v>17</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>129</v>
+        <v>186</v>
       </c>
       <c r="F13" t="s" s="0">
         <v>130</v>
@@ -1155,7 +1254,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
       </c>
     </row>
     <row r="14">
@@ -1172,7 +1271,7 @@
         <v>17</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>34</v>
+        <v>187</v>
       </c>
       <c r="F14" t="s" s="0">
         <v>35</v>
@@ -1199,18 +1298,62 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>167</v>
+        <v>175</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>189</v>
+      </c>
+      <c r="F15" t="s" s="0">
+        <v>190</v>
+      </c>
+      <c r="G15" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H15" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I15" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J15" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K15" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L15" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M15" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="N15" t="s" s="0">
+        <v>175</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N14"/>
+  <autoFilter ref="A1:N15"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C70"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1254,7 +1397,7 @@
         <v>43</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>73</v>
+        <v>191</v>
       </c>
     </row>
     <row r="5">
@@ -1298,7 +1441,7 @@
         <v>79</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>80</v>
+        <v>192</v>
       </c>
     </row>
     <row r="9">
@@ -1309,7 +1452,7 @@
         <v>81</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>82</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10">
@@ -1331,7 +1474,7 @@
         <v>41</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>91</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12">
@@ -1342,7 +1485,7 @@
         <v>43</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>92</v>
+        <v>195</v>
       </c>
     </row>
     <row r="13">
@@ -1529,7 +1672,7 @@
         <v>41</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>170</v>
+        <v>196</v>
       </c>
     </row>
     <row r="30">
@@ -1540,7 +1683,7 @@
         <v>43</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>171</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31">
@@ -1639,7 +1782,7 @@
         <v>43</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>44</v>
+        <v>198</v>
       </c>
     </row>
     <row r="40">
@@ -1694,7 +1837,7 @@
         <v>43</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>51</v>
+        <v>199</v>
       </c>
     </row>
     <row r="45">
@@ -1903,7 +2046,7 @@
         <v>43</v>
       </c>
       <c r="C63" t="s" s="0">
-        <v>61</v>
+        <v>200</v>
       </c>
     </row>
     <row r="64">
@@ -1928,8 +2071,63 @@
         <v>63</v>
       </c>
     </row>
+    <row r="66">
+      <c r="A66" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C66" t="s" s="0">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C67" t="s" s="0">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>203</v>
+      </c>
+      <c r="C68" t="s" s="0">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C69" t="s" s="0">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s" s="0">
+        <v>188</v>
+      </c>
+      <c r="B70" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C70" t="s" s="0">
+        <v>206</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C65"/>
+  <autoFilter ref="A1:C70"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh realm SQL state, drift reports, and CI artifacts
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4796" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5688" uniqueCount="236">
   <si>
     <t>candidate_id</t>
   </si>
@@ -719,6 +719,12 @@
   </si>
   <si>
     <t>775</t>
+  </si>
+  <si>
+    <t>2026-02-19T01:22:24Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T01:29:08Z</t>
   </si>
 </sst>
 </file>
@@ -851,7 +857,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="3">
@@ -895,7 +901,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="4">
@@ -939,7 +945,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="5">
@@ -983,7 +989,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="6">
@@ -1027,7 +1033,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="7">
@@ -1071,7 +1077,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8">
@@ -1115,7 +1121,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9">
@@ -1159,7 +1165,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="10">
@@ -1203,7 +1209,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11">
@@ -1247,7 +1253,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="12">
@@ -1291,7 +1297,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13">
@@ -1335,7 +1341,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14">
@@ -1379,7 +1385,7 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="15">
@@ -1423,7 +1429,7 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16">
@@ -1467,7 +1473,7 @@
         <v>89</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>208</v>
+        <v>235</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pm: complete queue-normalization pass with strict knowledge-link gating
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$18</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$86</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6186" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6710" uniqueCount="277">
   <si>
     <t>candidate_id</t>
   </si>
@@ -824,6 +824,30 @@
   </si>
   <si>
     <t>1348</t>
+  </si>
+  <si>
+    <t>2026-02-19T18:54:07Z</t>
+  </si>
+  <si>
+    <t>2026-02-19-queue-normalization-knowledge-link-gate</t>
+  </si>
+  <si>
+    <t>2026-02-19T18:52:55.836647834Z</t>
+  </si>
+  <si>
+    <t>Promote a high-leverage PM cycle that:</t>
+  </si>
+  <si>
+    <t>594</t>
+  </si>
+  <si>
+    <t>343</t>
+  </si>
+  <si>
+    <t>190</t>
+  </si>
+  <si>
+    <t>1682</t>
   </si>
 </sst>
 </file>
@@ -868,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -956,7 +980,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3">
@@ -1000,7 +1024,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4">
@@ -1044,7 +1068,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5">
@@ -1088,7 +1112,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6">
@@ -1132,7 +1156,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7">
@@ -1176,7 +1200,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8">
@@ -1220,7 +1244,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9">
@@ -1264,7 +1288,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10">
@@ -1308,7 +1332,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11">
@@ -1352,7 +1376,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12">
@@ -1396,7 +1420,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13">
@@ -1440,7 +1464,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14">
@@ -1484,7 +1508,7 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15">
@@ -1528,7 +1552,7 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16">
@@ -1572,7 +1596,7 @@
         <v>89</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17">
@@ -1616,15 +1640,15 @@
         <v>255</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>237</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="C18" t="s" s="0">
         <v>16</v>
@@ -1633,13 +1657,13 @@
         <v>17</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="G18" t="s" s="0">
-        <v>259</v>
+        <v>22</v>
       </c>
       <c r="H18" t="s" s="0">
         <v>108</v>
@@ -1657,21 +1681,65 @@
         <v>23</v>
       </c>
       <c r="M18" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="N18" t="s" s="0">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>257</v>
+      </c>
+      <c r="F19" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="G19" t="s" s="0">
+        <v>259</v>
+      </c>
+      <c r="H19" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I19" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J19" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K19" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L19" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M19" t="s" s="0">
         <v>260</v>
       </c>
-      <c r="N18" t="s" s="0">
-        <v>237</v>
+      <c r="N19" t="s" s="0">
+        <v>269</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N18"/>
+  <autoFilter ref="A1:N19"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C86"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2534,50 +2602,94 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B79" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>265</v>
+        <v>273</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B80" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C80" t="s" s="0">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B81" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C81" t="s" s="0">
-        <v>267</v>
+        <v>275</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B82" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C82" t="s" s="0">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C83" t="s" s="0">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C84" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C85" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C86" t="s" s="0">
         <v>268</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C82"/>
+  <autoFilter ref="A1:C86"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
pm: enforce human-friendly presentation refs and console id modes
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$90</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6710" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7260" uniqueCount="285">
   <si>
     <t>candidate_id</t>
   </si>
@@ -848,6 +848,30 @@
   </si>
   <si>
     <t>1682</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:22:43Z</t>
+  </si>
+  <si>
+    <t>2026-02-19-presentation-naming-governance-rollup</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:22:29.691767647Z</t>
+  </si>
+  <si>
+    <t>Standardize human-friendly presentation references for governance/decision/action/knowledge/release outputs while preserving internal IDs as storage/join keys.</t>
+  </si>
+  <si>
+    <t>641</t>
+  </si>
+  <si>
+    <t>240</t>
+  </si>
+  <si>
+    <t>270</t>
+  </si>
+  <si>
+    <t>1159</t>
   </si>
 </sst>
 </file>
@@ -892,7 +916,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -980,7 +1004,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="3">
@@ -1024,7 +1048,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="4">
@@ -1068,7 +1092,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="5">
@@ -1112,7 +1136,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="6">
@@ -1156,7 +1180,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="7">
@@ -1200,7 +1224,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8">
@@ -1244,7 +1268,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9">
@@ -1288,7 +1312,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10">
@@ -1332,7 +1356,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11">
@@ -1376,7 +1400,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12">
@@ -1420,7 +1444,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13">
@@ -1464,7 +1488,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14">
@@ -1508,7 +1532,7 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15">
@@ -1552,7 +1576,7 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16">
@@ -1596,7 +1620,7 @@
         <v>89</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17">
@@ -1640,15 +1664,15 @@
         <v>255</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="C18" t="s" s="0">
         <v>16</v>
@@ -1657,10 +1681,10 @@
         <v>17</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="G18" t="s" s="0">
         <v>22</v>
@@ -1681,18 +1705,18 @@
         <v>23</v>
       </c>
       <c r="M18" t="s" s="0">
-        <v>160</v>
+        <v>260</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>269</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="C19" t="s" s="0">
         <v>16</v>
@@ -1701,13 +1725,13 @@
         <v>17</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>257</v>
+        <v>271</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="G19" t="s" s="0">
-        <v>259</v>
+        <v>22</v>
       </c>
       <c r="H19" t="s" s="0">
         <v>108</v>
@@ -1725,21 +1749,65 @@
         <v>23</v>
       </c>
       <c r="M19" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="N19" t="s" s="0">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>257</v>
+      </c>
+      <c r="F20" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="G20" t="s" s="0">
+        <v>259</v>
+      </c>
+      <c r="H20" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I20" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J20" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K20" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L20" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M20" t="s" s="0">
         <v>260</v>
       </c>
-      <c r="N19" t="s" s="0">
-        <v>269</v>
+      <c r="N20" t="s" s="0">
+        <v>277</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N19"/>
+  <autoFilter ref="A1:N20"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C90"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2602,94 +2670,138 @@
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B79" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B80" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C80" t="s" s="0">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B81" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C81" t="s" s="0">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B82" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C82" t="s" s="0">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B83" t="s" s="0">
         <v>39</v>
       </c>
       <c r="C83" t="s" s="0">
-        <v>265</v>
+        <v>273</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B84" t="s" s="0">
         <v>41</v>
       </c>
       <c r="C84" t="s" s="0">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B85" t="s" s="0">
         <v>43</v>
       </c>
       <c r="C85" t="s" s="0">
-        <v>267</v>
+        <v>275</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B86" t="s" s="0">
         <v>45</v>
       </c>
       <c r="C86" t="s" s="0">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B87" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C87" t="s" s="0">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C88" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C89" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C90" t="s" s="0">
         <v>268</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C86"/>
+  <autoFilter ref="A1:C90"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
pm: persist all generated identifiers across disciplines in SQL registry
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7260" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7810" uniqueCount="287">
   <si>
     <t>candidate_id</t>
   </si>
@@ -872,6 +872,12 @@
   </si>
   <si>
     <t>1159</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:39:09Z</t>
+  </si>
+  <si>
+    <t>861</t>
   </si>
 </sst>
 </file>
@@ -1004,7 +1010,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3">
@@ -1048,7 +1054,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4">
@@ -1092,7 +1098,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="5">
@@ -1136,7 +1142,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6">
@@ -1180,7 +1186,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7">
@@ -1224,7 +1230,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="8">
@@ -1268,7 +1274,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9">
@@ -1312,7 +1318,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="10">
@@ -1356,7 +1362,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11">
@@ -1400,7 +1406,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="12">
@@ -1444,7 +1450,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13">
@@ -1488,7 +1494,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14">
@@ -1532,7 +1538,7 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="15">
@@ -1576,7 +1582,7 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="16">
@@ -1620,7 +1626,7 @@
         <v>89</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="17">
@@ -1664,7 +1670,7 @@
         <v>255</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18">
@@ -1708,7 +1714,7 @@
         <v>260</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19">
@@ -1752,7 +1758,7 @@
         <v>160</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20">
@@ -1796,7 +1802,7 @@
         <v>260</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
   </sheetData>
@@ -2676,7 +2682,7 @@
         <v>39</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>281</v>
+        <v>286</v>
       </c>
     </row>
     <row r="80">

</xml_diff>

<commit_message>
pm: automate delete-and-remanifest drill with safety gates and CI schedule
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7810" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8910" uniqueCount="309">
   <si>
     <t>candidate_id</t>
   </si>
@@ -878,6 +878,72 @@
   </si>
   <si>
     <t>861</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.611648835Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:48Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.602120753Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.605658836Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.604917128Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.612397918Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.609505627Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.607097419Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.607763919Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.604178378Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.597217587Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.608789585Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.598670003Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.606399253Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.613435877Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.600875545Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.599409712Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.600091211Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.602982836Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:45:26.597973628Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:46:37Z</t>
+  </si>
+  <si>
+    <t>1083</t>
   </si>
 </sst>
 </file>
@@ -983,7 +1049,7 @@
         <v>17</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>236</v>
+        <v>287</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>67</v>
@@ -1010,7 +1076,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3">
@@ -1027,7 +1093,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>238</v>
+        <v>289</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>87</v>
@@ -1054,7 +1120,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4">
@@ -1071,7 +1137,7 @@
         <v>17</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>239</v>
+        <v>290</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>124</v>
@@ -1098,7 +1164,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="5">
@@ -1115,7 +1181,7 @@
         <v>17</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>240</v>
+        <v>291</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>116</v>
@@ -1142,7 +1208,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="6">
@@ -1159,7 +1225,7 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>241</v>
+        <v>292</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>151</v>
@@ -1186,7 +1252,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="7">
@@ -1203,7 +1269,7 @@
         <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>242</v>
+        <v>293</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>159</v>
@@ -1230,7 +1296,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="8">
@@ -1247,7 +1313,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>243</v>
+        <v>294</v>
       </c>
       <c r="F8" t="s" s="0">
         <v>136</v>
@@ -1274,7 +1340,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="9">
@@ -1291,7 +1357,7 @@
         <v>17</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>244</v>
+        <v>295</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>19</v>
@@ -1318,7 +1384,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="10">
@@ -1335,7 +1401,7 @@
         <v>17</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>245</v>
+        <v>296</v>
       </c>
       <c r="F10" t="s" s="0">
         <v>29</v>
@@ -1362,7 +1428,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="11">
@@ -1379,7 +1445,7 @@
         <v>17</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>246</v>
+        <v>297</v>
       </c>
       <c r="F11" t="s" s="0">
         <v>107</v>
@@ -1406,7 +1472,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="12">
@@ -1423,7 +1489,7 @@
         <v>17</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>247</v>
+        <v>298</v>
       </c>
       <c r="F12" t="s" s="0">
         <v>143</v>
@@ -1450,7 +1516,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="13">
@@ -1467,7 +1533,7 @@
         <v>17</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>248</v>
+        <v>299</v>
       </c>
       <c r="F13" t="s" s="0">
         <v>130</v>
@@ -1494,7 +1560,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="14">
@@ -1511,7 +1577,7 @@
         <v>17</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>249</v>
+        <v>300</v>
       </c>
       <c r="F14" t="s" s="0">
         <v>35</v>
@@ -1538,7 +1604,7 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="15">
@@ -1555,7 +1621,7 @@
         <v>17</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>250</v>
+        <v>301</v>
       </c>
       <c r="F15" t="s" s="0">
         <v>190</v>
@@ -1582,7 +1648,7 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="16">
@@ -1599,7 +1665,7 @@
         <v>17</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>251</v>
+        <v>302</v>
       </c>
       <c r="F16" t="s" s="0">
         <v>224</v>
@@ -1626,7 +1692,7 @@
         <v>89</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17">
@@ -1643,7 +1709,7 @@
         <v>17</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>253</v>
+        <v>303</v>
       </c>
       <c r="F17" t="s" s="0">
         <v>254</v>
@@ -1670,7 +1736,7 @@
         <v>255</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18">
@@ -1687,7 +1753,7 @@
         <v>17</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>279</v>
+        <v>304</v>
       </c>
       <c r="F18" t="s" s="0">
         <v>280</v>
@@ -1714,7 +1780,7 @@
         <v>260</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="19">
@@ -1731,7 +1797,7 @@
         <v>17</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>271</v>
+        <v>305</v>
       </c>
       <c r="F19" t="s" s="0">
         <v>272</v>
@@ -1758,7 +1824,7 @@
         <v>160</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
     <row r="20">
@@ -1775,7 +1841,7 @@
         <v>17</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>257</v>
+        <v>306</v>
       </c>
       <c r="F20" t="s" s="0">
         <v>258</v>
@@ -1802,7 +1868,7 @@
         <v>260</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>285</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -2682,7 +2748,7 @@
         <v>39</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>286</v>
+        <v>308</v>
       </c>
     </row>
     <row r="80">

</xml_diff>

<commit_message>
Implement environment governance sprint tasks and validations
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$92</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8910" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9480" uniqueCount="333">
   <si>
     <t>candidate_id</t>
   </si>
@@ -944,6 +944,78 @@
   </si>
   <si>
     <t>1083</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.333131568Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T20:40:08Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.324442652Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.327982402Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.32722036Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.333922526Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.33180461Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.329531152Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.330346902Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.326483402Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.318863195Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.33107911Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.320688611Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.328820735Z</t>
+  </si>
+  <si>
+    <t>2026-02-19-console-environment-governance-v2</t>
+  </si>
+  <si>
+    <t>2026-02-19T20:23:39.04092028Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.334898068Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.323405319Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.321594694Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.322513944Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.325276777Z</t>
+  </si>
+  <si>
+    <t>2026-02-19T19:51:23.319735486Z</t>
+  </si>
+  <si>
+    <t>359</t>
+  </si>
+  <si>
+    <t>1130</t>
   </si>
 </sst>
 </file>
@@ -988,7 +1060,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N20"/>
+  <dimension ref="A1:N21"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1049,7 +1121,7 @@
         <v>17</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>287</v>
+        <v>309</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>67</v>
@@ -1076,7 +1148,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="3">
@@ -1093,7 +1165,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>289</v>
+        <v>311</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>87</v>
@@ -1120,7 +1192,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="4">
@@ -1137,7 +1209,7 @@
         <v>17</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>290</v>
+        <v>312</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>124</v>
@@ -1164,7 +1236,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="5">
@@ -1181,7 +1253,7 @@
         <v>17</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>291</v>
+        <v>313</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>116</v>
@@ -1208,7 +1280,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="6">
@@ -1225,7 +1297,7 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>292</v>
+        <v>314</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>151</v>
@@ -1252,7 +1324,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7">
@@ -1269,7 +1341,7 @@
         <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>293</v>
+        <v>315</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>159</v>
@@ -1296,7 +1368,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="8">
@@ -1313,7 +1385,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>294</v>
+        <v>316</v>
       </c>
       <c r="F8" t="s" s="0">
         <v>136</v>
@@ -1340,7 +1412,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="9">
@@ -1357,7 +1429,7 @@
         <v>17</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>295</v>
+        <v>317</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>19</v>
@@ -1384,7 +1456,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="10">
@@ -1401,7 +1473,7 @@
         <v>17</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>296</v>
+        <v>318</v>
       </c>
       <c r="F10" t="s" s="0">
         <v>29</v>
@@ -1428,7 +1500,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="11">
@@ -1445,7 +1517,7 @@
         <v>17</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>297</v>
+        <v>319</v>
       </c>
       <c r="F11" t="s" s="0">
         <v>107</v>
@@ -1472,7 +1544,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="12">
@@ -1489,7 +1561,7 @@
         <v>17</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>298</v>
+        <v>320</v>
       </c>
       <c r="F12" t="s" s="0">
         <v>143</v>
@@ -1516,7 +1588,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13">
@@ -1533,7 +1605,7 @@
         <v>17</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>299</v>
+        <v>321</v>
       </c>
       <c r="F13" t="s" s="0">
         <v>130</v>
@@ -1560,7 +1632,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14">
@@ -1577,7 +1649,7 @@
         <v>17</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>300</v>
+        <v>322</v>
       </c>
       <c r="F14" t="s" s="0">
         <v>35</v>
@@ -1604,15 +1676,15 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>188</v>
+        <v>323</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>188</v>
+        <v>323</v>
       </c>
       <c r="C15" t="s" s="0">
         <v>16</v>
@@ -1621,10 +1693,10 @@
         <v>17</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>301</v>
+        <v>324</v>
       </c>
       <c r="F15" t="s" s="0">
-        <v>190</v>
+        <v>22</v>
       </c>
       <c r="G15" t="s" s="0">
         <v>22</v>
@@ -1648,15 +1720,15 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="C16" t="s" s="0">
         <v>16</v>
@@ -1665,10 +1737,10 @@
         <v>17</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>302</v>
+        <v>325</v>
       </c>
       <c r="F16" t="s" s="0">
-        <v>224</v>
+        <v>190</v>
       </c>
       <c r="G16" t="s" s="0">
         <v>22</v>
@@ -1689,18 +1761,18 @@
         <v>23</v>
       </c>
       <c r="M16" t="s" s="0">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>252</v>
+        <v>222</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>252</v>
+        <v>222</v>
       </c>
       <c r="C17" t="s" s="0">
         <v>16</v>
@@ -1709,10 +1781,10 @@
         <v>17</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>303</v>
+        <v>326</v>
       </c>
       <c r="F17" t="s" s="0">
-        <v>254</v>
+        <v>224</v>
       </c>
       <c r="G17" t="s" s="0">
         <v>22</v>
@@ -1733,18 +1805,18 @@
         <v>23</v>
       </c>
       <c r="M17" t="s" s="0">
-        <v>255</v>
+        <v>89</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>278</v>
+        <v>252</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>278</v>
+        <v>252</v>
       </c>
       <c r="C18" t="s" s="0">
         <v>16</v>
@@ -1753,10 +1825,10 @@
         <v>17</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>304</v>
+        <v>327</v>
       </c>
       <c r="F18" t="s" s="0">
-        <v>280</v>
+        <v>254</v>
       </c>
       <c r="G18" t="s" s="0">
         <v>22</v>
@@ -1777,18 +1849,18 @@
         <v>23</v>
       </c>
       <c r="M18" t="s" s="0">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="C19" t="s" s="0">
         <v>16</v>
@@ -1797,10 +1869,10 @@
         <v>17</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>305</v>
+        <v>328</v>
       </c>
       <c r="F19" t="s" s="0">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="G19" t="s" s="0">
         <v>22</v>
@@ -1821,18 +1893,18 @@
         <v>23</v>
       </c>
       <c r="M19" t="s" s="0">
-        <v>160</v>
+        <v>260</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>307</v>
+        <v>310</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="C20" t="s" s="0">
         <v>16</v>
@@ -1841,13 +1913,13 @@
         <v>17</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>306</v>
+        <v>329</v>
       </c>
       <c r="F20" t="s" s="0">
-        <v>258</v>
+        <v>272</v>
       </c>
       <c r="G20" t="s" s="0">
-        <v>259</v>
+        <v>22</v>
       </c>
       <c r="H20" t="s" s="0">
         <v>108</v>
@@ -1865,21 +1937,65 @@
         <v>23</v>
       </c>
       <c r="M20" t="s" s="0">
+        <v>160</v>
+      </c>
+      <c r="N20" t="s" s="0">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>330</v>
+      </c>
+      <c r="F21" t="s" s="0">
+        <v>258</v>
+      </c>
+      <c r="G21" t="s" s="0">
+        <v>259</v>
+      </c>
+      <c r="H21" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I21" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J21" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K21" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L21" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M21" t="s" s="0">
         <v>260</v>
       </c>
-      <c r="N20" t="s" s="0">
-        <v>307</v>
+      <c r="N21" t="s" s="0">
+        <v>310</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N20"/>
+  <autoFilter ref="A1:N21"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C90"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -2599,24 +2715,24 @@
     </row>
     <row r="66">
       <c r="A66" t="s" s="0">
-        <v>188</v>
+        <v>323</v>
       </c>
       <c r="B66" t="s" s="0">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C66" t="s" s="0">
-        <v>201</v>
+        <v>331</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="s" s="0">
-        <v>188</v>
+        <v>323</v>
       </c>
       <c r="B67" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C67" t="s" s="0">
-        <v>202</v>
+        <v>332</v>
       </c>
     </row>
     <row r="68">
@@ -2624,10 +2740,10 @@
         <v>188</v>
       </c>
       <c r="B68" t="s" s="0">
-        <v>203</v>
+        <v>39</v>
       </c>
       <c r="C68" t="s" s="0">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="69">
@@ -2635,10 +2751,10 @@
         <v>188</v>
       </c>
       <c r="B69" t="s" s="0">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C69" t="s" s="0">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="70">
@@ -2646,32 +2762,32 @@
         <v>188</v>
       </c>
       <c r="B70" t="s" s="0">
-        <v>45</v>
+        <v>203</v>
       </c>
       <c r="C70" t="s" s="0">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="s" s="0">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="B71" t="s" s="0">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C71" t="s" s="0">
-        <v>230</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="s" s="0">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="B72" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C72" t="s" s="0">
-        <v>231</v>
+        <v>206</v>
       </c>
     </row>
     <row r="73">
@@ -2679,10 +2795,10 @@
         <v>222</v>
       </c>
       <c r="B73" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C73" t="s" s="0">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="74">
@@ -2690,32 +2806,32 @@
         <v>222</v>
       </c>
       <c r="B74" t="s" s="0">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C74" t="s" s="0">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="s" s="0">
-        <v>252</v>
+        <v>222</v>
       </c>
       <c r="B75" t="s" s="0">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C75" t="s" s="0">
-        <v>261</v>
+        <v>232</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="s" s="0">
-        <v>252</v>
+        <v>222</v>
       </c>
       <c r="B76" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C76" t="s" s="0">
-        <v>262</v>
+        <v>233</v>
       </c>
     </row>
     <row r="77">
@@ -2723,10 +2839,10 @@
         <v>252</v>
       </c>
       <c r="B77" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C77" t="s" s="0">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="78">
@@ -2734,32 +2850,32 @@
         <v>252</v>
       </c>
       <c r="B78" t="s" s="0">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C78" t="s" s="0">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="s" s="0">
-        <v>278</v>
+        <v>252</v>
       </c>
       <c r="B79" t="s" s="0">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C79" t="s" s="0">
-        <v>308</v>
+        <v>263</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="s" s="0">
-        <v>278</v>
+        <v>252</v>
       </c>
       <c r="B80" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C80" t="s" s="0">
-        <v>282</v>
+        <v>264</v>
       </c>
     </row>
     <row r="81">
@@ -2767,10 +2883,10 @@
         <v>278</v>
       </c>
       <c r="B81" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C81" t="s" s="0">
-        <v>283</v>
+        <v>308</v>
       </c>
     </row>
     <row r="82">
@@ -2778,32 +2894,32 @@
         <v>278</v>
       </c>
       <c r="B82" t="s" s="0">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C82" t="s" s="0">
-        <v>284</v>
+        <v>282</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B83" t="s" s="0">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C83" t="s" s="0">
-        <v>273</v>
+        <v>283</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="s" s="0">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="B84" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C84" t="s" s="0">
-        <v>274</v>
+        <v>284</v>
       </c>
     </row>
     <row r="85">
@@ -2811,10 +2927,10 @@
         <v>270</v>
       </c>
       <c r="B85" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C85" t="s" s="0">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="86">
@@ -2822,32 +2938,32 @@
         <v>270</v>
       </c>
       <c r="B86" t="s" s="0">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="C86" t="s" s="0">
-        <v>276</v>
+        <v>274</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B87" t="s" s="0">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C87" t="s" s="0">
-        <v>265</v>
+        <v>275</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="s" s="0">
-        <v>256</v>
+        <v>270</v>
       </c>
       <c r="B88" t="s" s="0">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C88" t="s" s="0">
-        <v>266</v>
+        <v>276</v>
       </c>
     </row>
     <row r="89">
@@ -2855,10 +2971,10 @@
         <v>256</v>
       </c>
       <c r="B89" t="s" s="0">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="C89" t="s" s="0">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="90">
@@ -2866,14 +2982,36 @@
         <v>256</v>
       </c>
       <c r="B90" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C90" t="s" s="0">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C91" t="s" s="0">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="s" s="0">
+        <v>256</v>
+      </c>
+      <c r="B92" t="s" s="0">
         <v>45</v>
       </c>
-      <c r="C90" t="s" s="0">
+      <c r="C92" t="s" s="0">
         <v>268</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C90"/>
+  <autoFilter ref="A1:C92"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
repo: finalize realm migration and strict environment-gate hardening
</commit_message>
<xml_diff>
--- a/docs/boilerplate-sync-candidates.xlsx
+++ b/docs/boilerplate-sync-candidates.xlsx
@@ -10,14 +10,14 @@
     <sheet name="Package Files" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Candidates!$A$1:$N$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">'Package Files'!$A$1:$C$96</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9480" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10672" uniqueCount="360">
   <si>
     <t>candidate_id</t>
   </si>
@@ -1016,6 +1016,87 @@
   </si>
   <si>
     <t>1130</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.383122224Z</t>
+  </si>
+  <si>
+    <t>2026-02-23T17:37:59Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.385297139Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.386419971Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.387527221Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.388373761Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.389769386Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.391086301Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.393768091Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.392442758Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.395207006Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.396273589Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.397223505Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.398216795Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.398897837Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.400493544Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.401785834Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.402773459Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.404318374Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.405822165Z</t>
+  </si>
+  <si>
+    <t>2026-02-20T01:46:01.408012246Z</t>
+  </si>
+  <si>
+    <t>2026-02-23-clean-recovery-alignment</t>
+  </si>
+  <si>
+    <t>2026-02-23T17:37:51.741916789Z</t>
+  </si>
+  <si>
+    <t>Describe what this package applies.</t>
+  </si>
+  <si>
+    <t>160</t>
+  </si>
+  <si>
+    <t>2026-02-23T17:49:05Z</t>
+  </si>
+  <si>
+    <t>976</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1141,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1121,7 +1202,7 @@
         <v>17</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>309</v>
+        <v>333</v>
       </c>
       <c r="F2" t="s" s="0">
         <v>67</v>
@@ -1148,7 +1229,7 @@
         <v>69</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="3">
@@ -1165,7 +1246,7 @@
         <v>17</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>311</v>
+        <v>335</v>
       </c>
       <c r="F3" t="s" s="0">
         <v>87</v>
@@ -1192,7 +1273,7 @@
         <v>31</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="4">
@@ -1209,7 +1290,7 @@
         <v>17</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>312</v>
+        <v>336</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>124</v>
@@ -1236,7 +1317,7 @@
         <v>89</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="5">
@@ -1253,7 +1334,7 @@
         <v>17</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>313</v>
+        <v>337</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>116</v>
@@ -1280,7 +1361,7 @@
         <v>31</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="6">
@@ -1297,7 +1378,7 @@
         <v>17</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>314</v>
+        <v>338</v>
       </c>
       <c r="F6" t="s" s="0">
         <v>151</v>
@@ -1324,7 +1405,7 @@
         <v>137</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="7">
@@ -1341,7 +1422,7 @@
         <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>315</v>
+        <v>339</v>
       </c>
       <c r="F7" t="s" s="0">
         <v>159</v>
@@ -1368,7 +1449,7 @@
         <v>168</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="8">
@@ -1385,7 +1466,7 @@
         <v>17</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="F8" t="s" s="0">
         <v>136</v>
@@ -1412,7 +1493,7 @@
         <v>137</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="9">
@@ -1429,7 +1510,7 @@
         <v>17</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="F9" t="s" s="0">
         <v>19</v>
@@ -1456,7 +1537,7 @@
         <v>24</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="10">
@@ -1473,7 +1554,7 @@
         <v>17</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>318</v>
+        <v>342</v>
       </c>
       <c r="F10" t="s" s="0">
         <v>29</v>
@@ -1500,7 +1581,7 @@
         <v>31</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="11">
@@ -1517,7 +1598,7 @@
         <v>17</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>319</v>
+        <v>343</v>
       </c>
       <c r="F11" t="s" s="0">
         <v>107</v>
@@ -1544,7 +1625,7 @@
         <v>89</v>
       </c>
       <c r="N11" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="12">
@@ -1561,7 +1642,7 @@
         <v>17</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>320</v>
+        <v>344</v>
       </c>
       <c r="F12" t="s" s="0">
         <v>143</v>
@@ -1588,7 +1669,7 @@
         <v>144</v>
       </c>
       <c r="N12" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="13">
@@ -1605,7 +1686,7 @@
         <v>17</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>321</v>
+        <v>345</v>
       </c>
       <c r="F13" t="s" s="0">
         <v>130</v>
@@ -1632,7 +1713,7 @@
         <v>89</v>
       </c>
       <c r="N13" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14">
@@ -1649,7 +1730,7 @@
         <v>17</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>322</v>
+        <v>346</v>
       </c>
       <c r="F14" t="s" s="0">
         <v>35</v>
@@ -1676,7 +1757,7 @@
         <v>24</v>
       </c>
       <c r="N14" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15">
@@ -1693,7 +1774,7 @@
         <v>17</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>324</v>
+        <v>347</v>
       </c>
       <c r="F15" t="s" s="0">
         <v>22</v>
@@ -1720,7 +1801,7 @@
         <v>108</v>
       </c>
       <c r="N15" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="16">
@@ -1737,7 +1818,7 @@
         <v>17</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>325</v>
+        <v>348</v>
       </c>
       <c r="F16" t="s" s="0">
         <v>190</v>
@@ -1764,7 +1845,7 @@
         <v>108</v>
       </c>
       <c r="N16" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="17">
@@ -1781,7 +1862,7 @@
         <v>17</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>326</v>
+        <v>349</v>
       </c>
       <c r="F17" t="s" s="0">
         <v>224</v>
@@ -1808,7 +1889,7 @@
         <v>89</v>
       </c>
       <c r="N17" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="18">
@@ -1825,7 +1906,7 @@
         <v>17</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>327</v>
+        <v>350</v>
       </c>
       <c r="F18" t="s" s="0">
         <v>254</v>
@@ -1852,7 +1933,7 @@
         <v>255</v>
       </c>
       <c r="N18" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="19">
@@ -1869,7 +1950,7 @@
         <v>17</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>328</v>
+        <v>351</v>
       </c>
       <c r="F19" t="s" s="0">
         <v>280</v>
@@ -1896,7 +1977,7 @@
         <v>260</v>
       </c>
       <c r="N19" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="20">
@@ -1913,7 +1994,7 @@
         <v>17</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>329</v>
+        <v>352</v>
       </c>
       <c r="F20" t="s" s="0">
         <v>272</v>
@@ -1940,7 +2021,7 @@
         <v>160</v>
       </c>
       <c r="N20" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
       </c>
     </row>
     <row r="21">
@@ -1957,7 +2038,7 @@
         <v>17</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>330</v>
+        <v>353</v>
       </c>
       <c r="F21" t="s" s="0">
         <v>258</v>
@@ -1984,18 +2065,62 @@
         <v>260</v>
       </c>
       <c r="N21" t="s" s="0">
-        <v>310</v>
+        <v>358</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>355</v>
+      </c>
+      <c r="F22" t="s" s="0">
+        <v>356</v>
+      </c>
+      <c r="G22" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="H22" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="I22" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J22" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="K22" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="L22" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="M22" t="s" s="0">
+        <v>108</v>
+      </c>
+      <c r="N22" t="s" s="0">
+        <v>358</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N21"/>
+  <autoFilter ref="A1:N22"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -3010,8 +3135,52 @@
         <v>268</v>
       </c>
     </row>
+    <row r="93">
+      <c r="A93" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="C93" t="s" s="0">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C94" t="s" s="0">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="B95" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C95" t="s" s="0">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="s" s="0">
+        <v>354</v>
+      </c>
+      <c r="B96" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C96" t="s" s="0">
+        <v>359</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C92"/>
+  <autoFilter ref="A1:C96"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>